<commit_message>
Updated datasets to latest results, retrained Liga MX models & fixed paths
</commit_message>
<xml_diff>
--- a/LigaMX/predictions/model_compareLMX.xlsx
+++ b/LigaMX/predictions/model_compareLMX.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\LigaMX\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34E5F6DC-9754-433C-A60C-4C80EC3A34BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04A0275B-02D8-4525-8E0E-C8234EBFF44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3264" yWindow="3264" windowWidth="17280" windowHeight="8904" activeTab="1" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
   <sheets>
     <sheet name="Models" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="60">
   <si>
     <t>Model</t>
   </si>
@@ -205,6 +205,18 @@
   </si>
   <si>
     <t>Santos Laguna Loss</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>model</t>
+  </si>
+  <si>
+    <t>cat_tune</t>
+  </si>
+  <si>
+    <t>lgbm_tune</t>
   </si>
 </sst>
 </file>
@@ -220,12 +232,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="12">
@@ -387,7 +405,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -423,6 +441,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -821,7 +841,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF436913-6699-4642-91DA-EC5EA358EA79}">
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="12.3671875" bestFit="1" customWidth="1"/>
@@ -885,31 +905,31 @@
         <v>7</v>
       </c>
       <c r="B3" s="1">
-        <v>0.6673</v>
+        <v>0.66959999999999997</v>
       </c>
       <c r="C3" s="1">
-        <v>0.47639999999999999</v>
+        <v>0.47820000000000001</v>
       </c>
       <c r="D3" s="1">
-        <v>0.68259999999999998</v>
+        <v>0.68310000000000004</v>
       </c>
       <c r="E3" s="1">
-        <v>0.4793</v>
+        <v>0.47870000000000001</v>
       </c>
       <c r="F3" s="1">
-        <v>0.69069999999999998</v>
+        <v>0.69669999999999999</v>
       </c>
       <c r="G3" s="3">
-        <v>0.48299999999999998</v>
+        <v>0.49030000000000001</v>
       </c>
       <c r="H3" s="4">
-        <v>0.75039999999999996</v>
+        <v>0.72309999999999997</v>
       </c>
       <c r="I3" s="1">
-        <v>0.57940000000000003</v>
+        <v>0.57420000000000004</v>
       </c>
       <c r="J3" s="5">
-        <v>0.60329999999999995</v>
+        <v>0.59140000000000004</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -917,31 +937,31 @@
         <v>6</v>
       </c>
       <c r="B4" s="1">
-        <v>0.66590000000000005</v>
+        <v>0.66410000000000002</v>
       </c>
       <c r="C4" s="1">
-        <v>0.4698</v>
+        <v>0.47089999999999999</v>
       </c>
       <c r="D4" s="1">
-        <v>0.66910000000000003</v>
+        <v>0.6694</v>
       </c>
       <c r="E4" s="1">
-        <v>0.48089999999999999</v>
+        <v>0.47899999999999998</v>
       </c>
       <c r="F4" s="1">
-        <v>0.6734</v>
+        <v>0.67589999999999995</v>
       </c>
       <c r="G4" s="3">
-        <v>0.47039999999999998</v>
+        <v>0.47049999999999997</v>
       </c>
       <c r="H4" s="4">
-        <v>0.7218</v>
+        <v>0.69479999999999997</v>
       </c>
       <c r="I4" s="1">
-        <v>0.57620000000000005</v>
+        <v>0.55459999999999998</v>
       </c>
       <c r="J4" s="5">
-        <v>0.5897</v>
+        <v>0.5726</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -949,31 +969,31 @@
         <v>8</v>
       </c>
       <c r="B5" s="1">
-        <v>0.66449999999999998</v>
+        <v>0.66569999999999996</v>
       </c>
       <c r="C5" s="1">
-        <v>0.47139999999999999</v>
+        <v>0.46879999999999999</v>
       </c>
       <c r="D5" s="1">
-        <v>0.67900000000000005</v>
+        <v>0.67949999999999999</v>
       </c>
       <c r="E5" s="1">
-        <v>0.4667</v>
+        <v>0.46379999999999999</v>
       </c>
       <c r="F5" s="1">
-        <v>0.6835</v>
+        <v>0.69030000000000002</v>
       </c>
       <c r="G5" s="3">
-        <v>0.48930000000000001</v>
+        <v>0.46229999999999999</v>
       </c>
       <c r="H5" s="4">
-        <v>0.745</v>
+        <v>0.72260000000000002</v>
       </c>
       <c r="I5" s="1">
-        <v>0.6008</v>
+        <v>0.50949999999999995</v>
       </c>
       <c r="J5" s="5">
-        <v>0.61140000000000005</v>
+        <v>0.58599999999999997</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -981,31 +1001,31 @@
         <v>5</v>
       </c>
       <c r="B6" s="1">
-        <v>0.66320000000000001</v>
+        <v>0.66510000000000002</v>
       </c>
       <c r="C6" s="1">
-        <v>0.46729999999999999</v>
+        <v>0.4798</v>
       </c>
       <c r="D6" s="1">
-        <v>0.67190000000000005</v>
+        <v>0.67400000000000004</v>
       </c>
       <c r="E6" s="1">
-        <v>0.44450000000000001</v>
+        <v>0.44890000000000002</v>
       </c>
       <c r="F6" s="1">
-        <v>0.6825</v>
+        <v>0.67369999999999997</v>
       </c>
       <c r="G6" s="3">
-        <v>0.44219999999999998</v>
+        <v>0.48399999999999999</v>
       </c>
       <c r="H6" s="4">
-        <v>0.73099999999999998</v>
+        <v>0.69669999999999999</v>
       </c>
       <c r="I6" s="1">
-        <v>0.58120000000000005</v>
+        <v>0.51739999999999997</v>
       </c>
       <c r="J6" s="5">
-        <v>0.60050000000000003</v>
+        <v>0.5403</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1013,31 +1033,31 @@
         <v>10</v>
       </c>
       <c r="B7" s="1">
-        <v>0.65549999999999997</v>
+        <v>0.65810000000000002</v>
       </c>
       <c r="C7" s="1">
-        <v>0.46479999999999999</v>
+        <v>0.4708</v>
       </c>
       <c r="D7" s="1">
-        <v>0.67920000000000003</v>
+        <v>0.67820000000000003</v>
       </c>
       <c r="E7" s="1">
-        <v>0.42580000000000001</v>
+        <v>0.42659999999999998</v>
       </c>
       <c r="F7" s="1">
-        <v>0.66830000000000001</v>
+        <v>0.66959999999999997</v>
       </c>
       <c r="G7" s="3">
-        <v>0.46939999999999998</v>
+        <v>0.47689999999999999</v>
       </c>
       <c r="H7" s="4">
-        <v>0.71930000000000005</v>
+        <v>0.69340000000000002</v>
       </c>
       <c r="I7" s="1">
-        <v>0.56379999999999997</v>
+        <v>0.53539999999999999</v>
       </c>
       <c r="J7" s="5">
-        <v>0.56520000000000004</v>
+        <v>0.53759999999999997</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1045,63 +1065,63 @@
         <v>11</v>
       </c>
       <c r="B8" s="1">
-        <v>0.65369999999999995</v>
+        <v>0.65490000000000004</v>
       </c>
       <c r="C8" s="1">
-        <v>0.45390000000000003</v>
+        <v>0.45519999999999999</v>
       </c>
       <c r="D8" s="1">
-        <v>0.63719999999999999</v>
+        <v>0.63759999999999994</v>
       </c>
       <c r="E8" s="1">
-        <v>0.41010000000000002</v>
+        <v>0.40860000000000002</v>
       </c>
       <c r="F8" s="1">
-        <v>0.66400000000000003</v>
+        <v>0.66620000000000001</v>
       </c>
       <c r="G8" s="3">
-        <v>0.4733</v>
+        <v>0.47699999999999998</v>
       </c>
       <c r="H8" s="4">
-        <v>0.73029999999999995</v>
+        <v>0.68540000000000001</v>
       </c>
       <c r="I8" s="1">
-        <v>0.57830000000000004</v>
+        <v>0.53320000000000001</v>
       </c>
       <c r="J8" s="5">
-        <v>0.5897</v>
+        <v>0.55110000000000003</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="18" t="s">
         <v>14</v>
       </c>
       <c r="B9" s="1">
-        <v>0.67630000000000001</v>
+        <v>0.68469999999999998</v>
       </c>
       <c r="C9" s="1">
-        <v>0.47949999999999998</v>
+        <v>0.4728</v>
       </c>
       <c r="D9" s="1">
-        <v>0.68179999999999996</v>
+        <v>0.68469999999999998</v>
       </c>
       <c r="E9" s="1">
-        <v>0.4834</v>
+        <v>0.47399999999999998</v>
       </c>
       <c r="F9" s="1">
-        <v>0.69399999999999995</v>
+        <v>0.69699999999999995</v>
       </c>
       <c r="G9" s="3">
-        <v>0.48709999999999998</v>
+        <v>0.47460000000000002</v>
       </c>
       <c r="H9" s="4">
-        <v>0.75470000000000004</v>
+        <v>0.72629999999999995</v>
       </c>
       <c r="I9" s="1">
-        <v>0.58550000000000002</v>
+        <v>0.55640000000000001</v>
       </c>
       <c r="J9" s="5">
-        <v>0.60599999999999998</v>
+        <v>0.5968</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1109,31 +1129,31 @@
         <v>17</v>
       </c>
       <c r="B10" s="1">
-        <v>0.68140000000000001</v>
+        <v>0.68159999999999998</v>
       </c>
       <c r="C10" s="1">
-        <v>0.48309999999999997</v>
+        <v>0.48580000000000001</v>
       </c>
       <c r="D10" s="1">
-        <v>0.67989999999999995</v>
+        <v>0.68020000000000003</v>
       </c>
       <c r="E10" s="1">
-        <v>0.4824</v>
+        <v>0.48759999999999998</v>
       </c>
       <c r="F10" s="1">
-        <v>0.68610000000000004</v>
+        <v>0.69199999999999995</v>
       </c>
       <c r="G10" s="3">
-        <v>0.47010000000000002</v>
+        <v>0.48759999999999998</v>
       </c>
       <c r="H10" s="4">
-        <v>0.74960000000000004</v>
+        <v>0.71750000000000003</v>
       </c>
       <c r="I10" s="1">
-        <v>0.58760000000000001</v>
+        <v>0.55600000000000005</v>
       </c>
       <c r="J10" s="5">
-        <v>0.61409999999999998</v>
+        <v>0.5806</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1141,31 +1161,31 @@
         <v>19</v>
       </c>
       <c r="B11" s="1">
-        <v>0.67120000000000002</v>
+        <v>0.67269999999999996</v>
       </c>
       <c r="C11" s="1">
-        <v>0.46139999999999998</v>
+        <v>0.4667</v>
       </c>
       <c r="D11" s="1">
-        <v>0.67979999999999996</v>
+        <v>0.68049999999999999</v>
       </c>
       <c r="E11" s="1">
-        <v>0.47499999999999998</v>
+        <v>0.4783</v>
       </c>
       <c r="F11" s="1">
-        <v>0.68910000000000005</v>
+        <v>0.69440000000000002</v>
       </c>
       <c r="G11" s="3">
-        <v>0.4743</v>
+        <v>0.48359999999999997</v>
       </c>
       <c r="H11" s="4">
-        <v>0.75439999999999996</v>
+        <v>0.72050000000000003</v>
       </c>
       <c r="I11" s="1">
-        <v>0.58950000000000002</v>
+        <v>0.56230000000000002</v>
       </c>
       <c r="J11" s="5">
-        <v>0.61680000000000001</v>
+        <v>0.58330000000000004</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1173,31 +1193,31 @@
         <v>18</v>
       </c>
       <c r="B12" s="1">
-        <v>0.67469999999999997</v>
+        <v>0.67600000000000005</v>
       </c>
       <c r="C12" s="1">
-        <v>0.4708</v>
+        <v>0.4738</v>
       </c>
       <c r="D12" s="1">
-        <v>0.68030000000000002</v>
+        <v>0.68240000000000001</v>
       </c>
       <c r="E12" s="1">
-        <v>0.47649999999999998</v>
+        <v>0.48420000000000002</v>
       </c>
       <c r="F12" s="1">
-        <v>0.68620000000000003</v>
+        <v>0.69510000000000005</v>
       </c>
       <c r="G12" s="3">
-        <v>0.4718</v>
+        <v>0.48220000000000002</v>
       </c>
       <c r="H12" s="4">
-        <v>0.753</v>
+        <v>0.71940000000000004</v>
       </c>
       <c r="I12" s="1">
-        <v>0.59279999999999999</v>
+        <v>0.56100000000000005</v>
       </c>
       <c r="J12" s="5">
-        <v>0.62229999999999996</v>
+        <v>0.5887</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1205,31 +1225,31 @@
         <v>20</v>
       </c>
       <c r="B13" s="1">
-        <v>0.67810000000000004</v>
+        <v>0.68400000000000005</v>
       </c>
       <c r="C13" s="1">
-        <v>0.47949999999999998</v>
+        <v>0.47870000000000001</v>
       </c>
       <c r="D13" s="1">
-        <v>0.68030000000000002</v>
+        <v>0.6845</v>
       </c>
       <c r="E13" s="1">
-        <v>0.48320000000000002</v>
+        <v>0.47399999999999998</v>
       </c>
       <c r="F13" s="1">
-        <v>0.69140000000000001</v>
+        <v>0.69540000000000002</v>
       </c>
       <c r="G13" s="3">
-        <v>0.48709999999999998</v>
+        <v>0.47670000000000001</v>
       </c>
       <c r="H13" s="4">
-        <v>0.75390000000000001</v>
+        <v>0.72199999999999998</v>
       </c>
       <c r="I13" s="1">
-        <v>0.5927</v>
+        <v>0.55769999999999997</v>
       </c>
       <c r="J13" s="5">
-        <v>0.62229999999999996</v>
+        <v>0.5968</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1237,31 +1257,31 @@
         <v>16</v>
       </c>
       <c r="B14" s="1">
-        <v>0.67120000000000002</v>
+        <v>0.67079999999999995</v>
       </c>
       <c r="C14" s="1">
-        <v>0.47310000000000002</v>
+        <v>0.4753</v>
       </c>
       <c r="D14" s="1">
-        <v>0.67130000000000001</v>
+        <v>0.67059999999999997</v>
       </c>
       <c r="E14" s="1">
-        <v>0.47189999999999999</v>
+        <v>0.4773</v>
       </c>
       <c r="F14" s="1">
-        <v>0.67520000000000002</v>
+        <v>0.68079999999999996</v>
       </c>
       <c r="G14" s="3">
-        <v>0.47670000000000001</v>
+        <v>0.47770000000000001</v>
       </c>
       <c r="H14" s="4">
-        <v>0.73429999999999995</v>
+        <v>0.70279999999999998</v>
       </c>
       <c r="I14" s="1">
-        <v>0.59689999999999999</v>
+        <v>0.56130000000000002</v>
       </c>
       <c r="J14" s="5">
-        <v>0.61409999999999998</v>
+        <v>0.58330000000000004</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1269,31 +1289,31 @@
         <v>15</v>
       </c>
       <c r="B15" s="1">
-        <v>0.66339999999999999</v>
+        <v>0.6714</v>
       </c>
       <c r="C15" s="1">
-        <v>0.46389999999999998</v>
+        <v>0.47649999999999998</v>
       </c>
       <c r="D15" s="1">
-        <v>0.66490000000000005</v>
+        <v>0.68010000000000004</v>
       </c>
       <c r="E15" s="1">
-        <v>0.4698</v>
+        <v>0.47510000000000002</v>
       </c>
       <c r="F15" s="1">
-        <v>0.68330000000000002</v>
+        <v>0.69110000000000005</v>
       </c>
       <c r="G15" s="3">
-        <v>0.48270000000000002</v>
+        <v>0.47289999999999999</v>
       </c>
       <c r="H15" s="4">
-        <v>0.74270000000000003</v>
+        <v>0.72260000000000002</v>
       </c>
       <c r="I15" s="1">
-        <v>0.59909999999999997</v>
+        <v>0.55569999999999997</v>
       </c>
       <c r="J15" s="5">
-        <v>0.60870000000000002</v>
+        <v>0.59409999999999996</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1301,31 +1321,31 @@
         <v>9</v>
       </c>
       <c r="B16" s="1">
-        <v>0.67669999999999997</v>
+        <v>0.68010000000000004</v>
       </c>
       <c r="C16" s="1">
-        <v>0.47520000000000001</v>
+        <v>0.48089999999999999</v>
       </c>
       <c r="D16" s="1">
-        <v>0.67869999999999997</v>
+        <v>0.68169999999999997</v>
       </c>
       <c r="E16" s="1">
-        <v>0.48120000000000002</v>
+        <v>0.48649999999999999</v>
       </c>
       <c r="F16" s="1">
-        <v>0.69140000000000001</v>
+        <v>0.69240000000000002</v>
       </c>
       <c r="G16" s="3">
-        <v>0.48099999999999998</v>
+        <v>0.47720000000000001</v>
       </c>
       <c r="H16" s="4">
-        <v>0.75139999999999996</v>
+        <v>0.71870000000000001</v>
       </c>
       <c r="I16" s="1">
-        <v>0.61360000000000003</v>
+        <v>0.5675</v>
       </c>
       <c r="J16" s="5">
-        <v>0.63039999999999996</v>
+        <v>0.5968</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1351,6 +1371,77 @@
       <c r="H18" s="6"/>
       <c r="I18" s="7"/>
       <c r="J18" s="8"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="B19" t="s">
+        <v>58</v>
+      </c>
+      <c r="C19" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" t="s">
+        <v>59</v>
+      </c>
+      <c r="E19" t="s">
+        <v>5</v>
+      </c>
+      <c r="F19" t="s">
+        <v>10</v>
+      </c>
+      <c r="G19" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="B20" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="B21" s="17">
+        <v>46128</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" s="1">
+        <v>0.75390000000000001</v>
+      </c>
+      <c r="E21" s="1">
+        <v>0.5927</v>
+      </c>
+      <c r="F21" s="1">
+        <v>0.62229999999999996</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="B22" s="17">
+        <v>46134</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0.72629999999999995</v>
+      </c>
+      <c r="E22" s="1">
+        <v>0.55640000000000001</v>
+      </c>
+      <c r="F22" s="1">
+        <v>0.5968</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1393,7 +1484,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2AB4D39-76AB-4A8D-8A49-E2E912416120}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="2" max="2" width="13.578125" bestFit="1" customWidth="1"/>
@@ -1571,6 +1662,51 @@
         <v>55</v>
       </c>
     </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated Liga MX data, retrained data and updated paths
</commit_message>
<xml_diff>
--- a/LigaMX/predictions/model_compareLMX.xlsx
+++ b/LigaMX/predictions/model_compareLMX.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\LigaMX\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04A0275B-02D8-4525-8E0E-C8234EBFF44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61060F73-0BFA-4077-857E-2071008BE5C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
+    <workbookView xWindow="-78" yWindow="0" windowWidth="11676" windowHeight="12318" activeTab="1" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
   <sheets>
     <sheet name="Models" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="69">
   <si>
     <t>Model</t>
   </si>
@@ -117,9 +117,6 @@
     <t>Pumas UNAM</t>
   </si>
   <si>
-    <t>San Luis Loss</t>
-  </si>
-  <si>
     <t>Mazatlan</t>
   </si>
   <si>
@@ -216,7 +213,37 @@
     <t>cat_tune</t>
   </si>
   <si>
-    <t>lgbm_tune</t>
+    <t>Pumas UNAM Win</t>
+  </si>
+  <si>
+    <t>Queretaro Loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leon </t>
+  </si>
+  <si>
+    <t>Leon Loss</t>
+  </si>
+  <si>
+    <t>Atlas Loss</t>
+  </si>
+  <si>
+    <t>Atletico San Luis Win</t>
+  </si>
+  <si>
+    <t>Atletico San Luis Loss</t>
+  </si>
+  <si>
+    <t>Mazatlan Loss</t>
+  </si>
+  <si>
+    <t>Tijuana Win</t>
+  </si>
+  <si>
+    <t>cat_xgb</t>
+  </si>
+  <si>
+    <t>cat_lgbm_xgb</t>
   </si>
 </sst>
 </file>
@@ -405,7 +432,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -443,6 +470,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -841,11 +869,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF436913-6699-4642-91DA-EC5EA358EA79}">
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="12.3671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="9.26171875" customWidth="1"/>
+    <col min="2" max="2" width="9.26171875" customWidth="1"/>
+    <col min="3" max="3" width="11.3125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="36.299999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -905,31 +934,31 @@
         <v>7</v>
       </c>
       <c r="B3" s="1">
-        <v>0.66959999999999997</v>
+        <v>0.66469999999999996</v>
       </c>
       <c r="C3" s="1">
-        <v>0.47820000000000001</v>
+        <v>0.47420000000000001</v>
       </c>
       <c r="D3" s="1">
-        <v>0.68310000000000004</v>
+        <v>0.68489999999999995</v>
       </c>
       <c r="E3" s="1">
-        <v>0.47870000000000001</v>
+        <v>0.47749999999999998</v>
       </c>
       <c r="F3" s="1">
-        <v>0.69669999999999999</v>
+        <v>0.70269999999999999</v>
       </c>
       <c r="G3" s="3">
-        <v>0.49030000000000001</v>
+        <v>0.50209999999999999</v>
       </c>
       <c r="H3" s="4">
-        <v>0.72309999999999997</v>
+        <v>0.70699999999999996</v>
       </c>
       <c r="I3" s="1">
-        <v>0.57420000000000004</v>
+        <v>0.5333</v>
       </c>
       <c r="J3" s="5">
-        <v>0.59140000000000004</v>
+        <v>0.57250000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -937,31 +966,31 @@
         <v>6</v>
       </c>
       <c r="B4" s="1">
-        <v>0.66410000000000002</v>
+        <v>0.6663</v>
       </c>
       <c r="C4" s="1">
-        <v>0.47089999999999999</v>
+        <v>0.4672</v>
       </c>
       <c r="D4" s="1">
-        <v>0.6694</v>
+        <v>0.6704</v>
       </c>
       <c r="E4" s="1">
-        <v>0.47899999999999998</v>
+        <v>0.4783</v>
       </c>
       <c r="F4" s="1">
-        <v>0.67589999999999995</v>
+        <v>0.68489999999999995</v>
       </c>
       <c r="G4" s="3">
-        <v>0.47049999999999997</v>
+        <v>0.49469999999999997</v>
       </c>
       <c r="H4" s="4">
-        <v>0.69479999999999997</v>
+        <v>0.68469999999999998</v>
       </c>
       <c r="I4" s="1">
-        <v>0.55459999999999998</v>
+        <v>0.52949999999999997</v>
       </c>
       <c r="J4" s="5">
-        <v>0.5726</v>
+        <v>0.56159999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -969,31 +998,31 @@
         <v>8</v>
       </c>
       <c r="B5" s="1">
-        <v>0.66569999999999996</v>
+        <v>0.66600000000000004</v>
       </c>
       <c r="C5" s="1">
-        <v>0.46879999999999999</v>
+        <v>0.47549999999999998</v>
       </c>
       <c r="D5" s="1">
-        <v>0.67949999999999999</v>
+        <v>0.67820000000000003</v>
       </c>
       <c r="E5" s="1">
-        <v>0.46379999999999999</v>
+        <v>0.46100000000000002</v>
       </c>
       <c r="F5" s="1">
-        <v>0.69030000000000002</v>
+        <v>0.69530000000000003</v>
       </c>
       <c r="G5" s="3">
-        <v>0.46229999999999999</v>
+        <v>0.46920000000000001</v>
       </c>
       <c r="H5" s="4">
-        <v>0.72260000000000002</v>
+        <v>0.7006</v>
       </c>
       <c r="I5" s="1">
-        <v>0.50949999999999995</v>
+        <v>0.54149999999999998</v>
       </c>
       <c r="J5" s="5">
-        <v>0.58599999999999997</v>
+        <v>0.55430000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1001,31 +1030,31 @@
         <v>5</v>
       </c>
       <c r="B6" s="1">
-        <v>0.66510000000000002</v>
+        <v>0.66439999999999999</v>
       </c>
       <c r="C6" s="1">
-        <v>0.4798</v>
+        <v>0.46779999999999999</v>
       </c>
       <c r="D6" s="1">
-        <v>0.67400000000000004</v>
+        <v>0.67300000000000004</v>
       </c>
       <c r="E6" s="1">
-        <v>0.44890000000000002</v>
+        <v>0.44579999999999997</v>
       </c>
       <c r="F6" s="1">
-        <v>0.67369999999999997</v>
+        <v>0.69230000000000003</v>
       </c>
       <c r="G6" s="3">
-        <v>0.48399999999999999</v>
+        <v>0.4521</v>
       </c>
       <c r="H6" s="4">
-        <v>0.69669999999999999</v>
+        <v>0.69850000000000001</v>
       </c>
       <c r="I6" s="1">
-        <v>0.51739999999999997</v>
+        <v>0.5131</v>
       </c>
       <c r="J6" s="5">
-        <v>0.5403</v>
+        <v>0.54349999999999998</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1033,31 +1062,31 @@
         <v>10</v>
       </c>
       <c r="B7" s="1">
-        <v>0.65810000000000002</v>
+        <v>0.65359999999999996</v>
       </c>
       <c r="C7" s="1">
-        <v>0.4708</v>
+        <v>0.45929999999999999</v>
       </c>
       <c r="D7" s="1">
-        <v>0.67820000000000003</v>
+        <v>0.67800000000000005</v>
       </c>
       <c r="E7" s="1">
-        <v>0.42659999999999998</v>
+        <v>0.42380000000000001</v>
       </c>
       <c r="F7" s="1">
-        <v>0.66959999999999997</v>
+        <v>0.67969999999999997</v>
       </c>
       <c r="G7" s="3">
-        <v>0.47689999999999999</v>
+        <v>0.48899999999999999</v>
       </c>
       <c r="H7" s="4">
-        <v>0.69340000000000002</v>
+        <v>0.69259999999999999</v>
       </c>
       <c r="I7" s="1">
-        <v>0.53539999999999999</v>
+        <v>0.53380000000000005</v>
       </c>
       <c r="J7" s="5">
-        <v>0.53759999999999997</v>
+        <v>0.54349999999999998</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1065,63 +1094,63 @@
         <v>11</v>
       </c>
       <c r="B8" s="1">
-        <v>0.65490000000000004</v>
+        <v>0.65559999999999996</v>
       </c>
       <c r="C8" s="1">
-        <v>0.45519999999999999</v>
+        <v>0.4577</v>
       </c>
       <c r="D8" s="1">
-        <v>0.63759999999999994</v>
+        <v>0.63839999999999997</v>
       </c>
       <c r="E8" s="1">
-        <v>0.40860000000000002</v>
+        <v>0.40939999999999999</v>
       </c>
       <c r="F8" s="1">
-        <v>0.66620000000000001</v>
+        <v>0.67359999999999998</v>
       </c>
       <c r="G8" s="3">
-        <v>0.47699999999999998</v>
+        <v>0.48380000000000001</v>
       </c>
       <c r="H8" s="4">
-        <v>0.68540000000000001</v>
+        <v>0.62990000000000002</v>
       </c>
       <c r="I8" s="1">
-        <v>0.53320000000000001</v>
+        <v>0.50470000000000004</v>
       </c>
       <c r="J8" s="5">
-        <v>0.55110000000000003</v>
+        <v>0.52900000000000003</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="19" t="s">
         <v>14</v>
       </c>
       <c r="B9" s="1">
-        <v>0.68469999999999998</v>
+        <v>0.67910000000000004</v>
       </c>
       <c r="C9" s="1">
-        <v>0.4728</v>
+        <v>0.47939999999999999</v>
       </c>
       <c r="D9" s="1">
-        <v>0.68469999999999998</v>
+        <v>0.68369999999999997</v>
       </c>
       <c r="E9" s="1">
-        <v>0.47399999999999998</v>
+        <v>0.47989999999999999</v>
       </c>
       <c r="F9" s="1">
-        <v>0.69699999999999995</v>
+        <v>0.70530000000000004</v>
       </c>
       <c r="G9" s="3">
-        <v>0.47460000000000002</v>
+        <v>0.49909999999999999</v>
       </c>
       <c r="H9" s="4">
-        <v>0.72629999999999995</v>
+        <v>0.71050000000000002</v>
       </c>
       <c r="I9" s="1">
-        <v>0.55640000000000001</v>
+        <v>0.55159999999999998</v>
       </c>
       <c r="J9" s="5">
-        <v>0.5968</v>
+        <v>0.58699999999999997</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1129,31 +1158,31 @@
         <v>17</v>
       </c>
       <c r="B10" s="1">
-        <v>0.68159999999999998</v>
+        <v>0.68340000000000001</v>
       </c>
       <c r="C10" s="1">
-        <v>0.48580000000000001</v>
+        <v>0.47789999999999999</v>
       </c>
       <c r="D10" s="1">
-        <v>0.68020000000000003</v>
+        <v>0.68189999999999995</v>
       </c>
       <c r="E10" s="1">
-        <v>0.48759999999999998</v>
+        <v>0.47870000000000001</v>
       </c>
       <c r="F10" s="1">
-        <v>0.69199999999999995</v>
+        <v>0.70240000000000002</v>
       </c>
       <c r="G10" s="3">
-        <v>0.48759999999999998</v>
+        <v>0.48399999999999999</v>
       </c>
       <c r="H10" s="4">
-        <v>0.71750000000000003</v>
+        <v>0.71089999999999998</v>
       </c>
       <c r="I10" s="1">
-        <v>0.55600000000000005</v>
+        <v>0.53710000000000002</v>
       </c>
       <c r="J10" s="5">
-        <v>0.5806</v>
+        <v>0.57609999999999995</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1161,31 +1190,31 @@
         <v>19</v>
       </c>
       <c r="B11" s="1">
-        <v>0.67269999999999996</v>
+        <v>0.67390000000000005</v>
       </c>
       <c r="C11" s="1">
-        <v>0.4667</v>
+        <v>0.46660000000000001</v>
       </c>
       <c r="D11" s="1">
-        <v>0.68049999999999999</v>
+        <v>0.68220000000000003</v>
       </c>
       <c r="E11" s="1">
-        <v>0.4783</v>
+        <v>0.47699999999999998</v>
       </c>
       <c r="F11" s="1">
-        <v>0.69440000000000002</v>
+        <v>0.70099999999999996</v>
       </c>
       <c r="G11" s="3">
-        <v>0.48359999999999997</v>
+        <v>0.48720000000000002</v>
       </c>
       <c r="H11" s="4">
-        <v>0.72050000000000003</v>
+        <v>0.68640000000000001</v>
       </c>
       <c r="I11" s="1">
-        <v>0.56230000000000002</v>
+        <v>0.49619999999999997</v>
       </c>
       <c r="J11" s="5">
-        <v>0.58330000000000004</v>
+        <v>0.53620000000000001</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1193,31 +1222,31 @@
         <v>18</v>
       </c>
       <c r="B12" s="1">
-        <v>0.67600000000000005</v>
+        <v>0.67730000000000001</v>
       </c>
       <c r="C12" s="1">
-        <v>0.4738</v>
+        <v>0.47160000000000002</v>
       </c>
       <c r="D12" s="1">
-        <v>0.68240000000000001</v>
+        <v>0.68269999999999997</v>
       </c>
       <c r="E12" s="1">
-        <v>0.48420000000000002</v>
+        <v>0.47899999999999998</v>
       </c>
       <c r="F12" s="1">
-        <v>0.69510000000000005</v>
+        <v>0.70179999999999998</v>
       </c>
       <c r="G12" s="3">
-        <v>0.48220000000000002</v>
+        <v>0.48749999999999999</v>
       </c>
       <c r="H12" s="4">
-        <v>0.71940000000000004</v>
+        <v>0.69750000000000001</v>
       </c>
       <c r="I12" s="1">
-        <v>0.56100000000000005</v>
+        <v>0.50270000000000004</v>
       </c>
       <c r="J12" s="5">
-        <v>0.5887</v>
+        <v>0.54710000000000003</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1225,31 +1254,31 @@
         <v>20</v>
       </c>
       <c r="B13" s="1">
-        <v>0.68400000000000005</v>
+        <v>0.68100000000000005</v>
       </c>
       <c r="C13" s="1">
-        <v>0.47870000000000001</v>
+        <v>0.47560000000000002</v>
       </c>
       <c r="D13" s="1">
-        <v>0.6845</v>
+        <v>0.68289999999999995</v>
       </c>
       <c r="E13" s="1">
-        <v>0.47399999999999998</v>
+        <v>0.47610000000000002</v>
       </c>
       <c r="F13" s="1">
-        <v>0.69540000000000002</v>
+        <v>0.70469999999999999</v>
       </c>
       <c r="G13" s="3">
-        <v>0.47670000000000001</v>
+        <v>0.49280000000000002</v>
       </c>
       <c r="H13" s="4">
-        <v>0.72199999999999998</v>
+        <v>0.71430000000000005</v>
       </c>
       <c r="I13" s="1">
-        <v>0.55769999999999997</v>
+        <v>0.5383</v>
       </c>
       <c r="J13" s="5">
-        <v>0.5968</v>
+        <v>0.57609999999999995</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1257,31 +1286,31 @@
         <v>16</v>
       </c>
       <c r="B14" s="1">
-        <v>0.67079999999999995</v>
+        <v>0.67249999999999999</v>
       </c>
       <c r="C14" s="1">
-        <v>0.4753</v>
+        <v>0.47239999999999999</v>
       </c>
       <c r="D14" s="1">
-        <v>0.67059999999999997</v>
+        <v>0.6724</v>
       </c>
       <c r="E14" s="1">
-        <v>0.4773</v>
+        <v>0.47889999999999999</v>
       </c>
       <c r="F14" s="1">
-        <v>0.68079999999999996</v>
+        <v>0.68640000000000001</v>
       </c>
       <c r="G14" s="3">
-        <v>0.47770000000000001</v>
+        <v>0.48599999999999999</v>
       </c>
       <c r="H14" s="4">
-        <v>0.70279999999999998</v>
+        <v>0.69969999999999999</v>
       </c>
       <c r="I14" s="1">
-        <v>0.56130000000000002</v>
+        <v>0.53700000000000003</v>
       </c>
       <c r="J14" s="5">
-        <v>0.58330000000000004</v>
+        <v>0.57250000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1289,31 +1318,31 @@
         <v>15</v>
       </c>
       <c r="B15" s="1">
-        <v>0.6714</v>
+        <v>0.66279999999999994</v>
       </c>
       <c r="C15" s="1">
-        <v>0.47649999999999998</v>
+        <v>0.47</v>
       </c>
       <c r="D15" s="1">
-        <v>0.68010000000000004</v>
+        <v>0.66479999999999995</v>
       </c>
       <c r="E15" s="1">
-        <v>0.47510000000000002</v>
+        <v>0.47260000000000002</v>
       </c>
       <c r="F15" s="1">
-        <v>0.69110000000000005</v>
+        <v>0.69320000000000004</v>
       </c>
       <c r="G15" s="3">
-        <v>0.47289999999999999</v>
+        <v>0.4985</v>
       </c>
       <c r="H15" s="4">
-        <v>0.72260000000000002</v>
+        <v>0.70379999999999998</v>
       </c>
       <c r="I15" s="1">
-        <v>0.55569999999999997</v>
+        <v>0.54790000000000005</v>
       </c>
       <c r="J15" s="5">
-        <v>0.59409999999999996</v>
+        <v>0.56159999999999999</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
@@ -1321,66 +1350,106 @@
         <v>9</v>
       </c>
       <c r="B16" s="1">
-        <v>0.68010000000000004</v>
+        <v>0.67810000000000004</v>
       </c>
       <c r="C16" s="1">
-        <v>0.48089999999999999</v>
+        <v>0.47370000000000001</v>
       </c>
       <c r="D16" s="1">
-        <v>0.68169999999999997</v>
+        <v>0.67720000000000002</v>
       </c>
       <c r="E16" s="1">
-        <v>0.48649999999999999</v>
+        <v>0.47689999999999999</v>
       </c>
       <c r="F16" s="1">
-        <v>0.69240000000000002</v>
+        <v>0.70140000000000002</v>
       </c>
       <c r="G16" s="3">
-        <v>0.47720000000000001</v>
+        <v>0.4909</v>
       </c>
       <c r="H16" s="4">
-        <v>0.71870000000000001</v>
+        <v>0.69820000000000004</v>
       </c>
       <c r="I16" s="1">
-        <v>0.5675</v>
+        <v>0.53549999999999998</v>
       </c>
       <c r="J16" s="5">
-        <v>0.5968</v>
+        <v>0.56159999999999999</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="5"/>
+      <c r="A17" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" s="1">
+        <v>0.67130000000000001</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0.46929999999999999</v>
+      </c>
+      <c r="D17" s="1">
+        <v>0.68049999999999999</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0.47989999999999999</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0.70389999999999997</v>
+      </c>
+      <c r="G17" s="3">
+        <v>0.49199999999999999</v>
+      </c>
+      <c r="H17" s="4">
+        <v>0.71260000000000001</v>
+      </c>
+      <c r="I17" s="1">
+        <v>0.54869999999999997</v>
+      </c>
+      <c r="J17" s="5">
+        <v>0.57250000000000001</v>
+      </c>
     </row>
     <row r="18" spans="1:10" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="7"/>
-      <c r="J18" s="8"/>
+      <c r="A18" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" s="1">
+        <v>0.67220000000000002</v>
+      </c>
+      <c r="C18" s="1">
+        <v>0.47249999999999998</v>
+      </c>
+      <c r="D18" s="1">
+        <v>0.6794</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.47649999999999998</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0.70430000000000004</v>
+      </c>
+      <c r="G18" s="3">
+        <v>0.4975</v>
+      </c>
+      <c r="H18" s="6">
+        <v>0.7127</v>
+      </c>
+      <c r="I18" s="7">
+        <v>0.56720000000000004</v>
+      </c>
+      <c r="J18" s="8">
+        <v>0.58699999999999997</v>
+      </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C19" t="s">
         <v>6</v>
       </c>
       <c r="D19" t="s">
-        <v>59</v>
+        <v>8</v>
       </c>
       <c r="E19" t="s">
         <v>5</v>
@@ -1394,10 +1463,10 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B20" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>12</v>
@@ -1428,7 +1497,7 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B22" s="9">
-        <v>46134</v>
+        <v>46131</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>14</v>
@@ -1441,6 +1510,23 @@
       </c>
       <c r="F22" s="1">
         <v>0.5968</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="B23" s="9">
+        <v>46135</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D23" s="1">
+        <v>0.7127</v>
+      </c>
+      <c r="E23" s="1">
+        <v>0.56720000000000004</v>
+      </c>
+      <c r="F23" s="1">
+        <v>0.58699999999999997</v>
       </c>
     </row>
   </sheetData>
@@ -1484,17 +1570,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2AB4D39-76AB-4A8D-8A49-E2E912416120}">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="2" max="2" width="13.578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.3671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="16.1015625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="13.578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="17.578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B1" t="s">
         <v>22</v>
@@ -1503,10 +1588,10 @@
         <v>23</v>
       </c>
       <c r="D1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" t="s">
         <v>42</v>
-      </c>
-      <c r="E1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1520,10 +1605,10 @@
         <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>64</v>
       </c>
       <c r="E2" t="s">
-        <v>26</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1531,16 +1616,16 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1548,16 +1633,16 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
         <v>30</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>31</v>
       </c>
-      <c r="D4" t="s">
-        <v>32</v>
-      </c>
       <c r="E4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1565,16 +1650,16 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
         <v>33</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>34</v>
       </c>
-      <c r="D5" t="s">
-        <v>35</v>
-      </c>
       <c r="E5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1582,16 +1667,16 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
         <v>36</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>37</v>
       </c>
-      <c r="D6" t="s">
-        <v>38</v>
-      </c>
       <c r="E6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1599,16 +1684,16 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
         <v>40</v>
       </c>
-      <c r="C7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" t="s">
-        <v>41</v>
-      </c>
       <c r="E7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1616,16 +1701,16 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" t="s">
         <v>44</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>45</v>
       </c>
-      <c r="D8" t="s">
-        <v>46</v>
-      </c>
       <c r="E8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1633,16 +1718,16 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" t="s">
         <v>50</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" t="s">
         <v>51</v>
-      </c>
-      <c r="D9" t="s">
-        <v>48</v>
-      </c>
-      <c r="E9" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1650,61 +1735,268 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" t="s">
         <v>53</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>54</v>
       </c>
-      <c r="D10" t="s">
-        <v>55</v>
-      </c>
       <c r="E10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A11">
         <v>16</v>
       </c>
+      <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A12">
         <v>16</v>
       </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E12" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A13">
         <v>16</v>
       </c>
+      <c r="B13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" t="s">
+        <v>37</v>
+      </c>
+      <c r="E13" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A14">
         <v>16</v>
       </c>
+      <c r="B14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A15">
         <v>16</v>
       </c>
+      <c r="B15" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" t="s">
+        <v>62</v>
+      </c>
+      <c r="E15" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A16">
         <v>16</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A17">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" t="s">
+        <v>65</v>
+      </c>
+      <c r="E17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A18">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B18" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A19">
         <v>16</v>
+      </c>
+      <c r="B19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" t="s">
+        <v>66</v>
+      </c>
+      <c r="E19" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20">
+        <v>17</v>
+      </c>
+      <c r="B20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21">
+        <v>17</v>
+      </c>
+      <c r="B21" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A22">
+        <v>17</v>
+      </c>
+      <c r="B22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A23">
+        <v>17</v>
+      </c>
+      <c r="B23" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A24">
+        <v>17</v>
+      </c>
+      <c r="B24" t="s">
+        <v>39</v>
+      </c>
+      <c r="C24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A25">
+        <v>17</v>
+      </c>
+      <c r="B25" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A26">
+        <v>17</v>
+      </c>
+      <c r="B26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A27">
+        <v>17</v>
+      </c>
+      <c r="B27" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A28">
+        <v>17</v>
+      </c>
+      <c r="B28" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated results page with end of the season results
</commit_message>
<xml_diff>
--- a/LigaMX/predictions/model_compareLMX.xlsx
+++ b/LigaMX/predictions/model_compareLMX.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ripa_\Desktop\Programing\IndyCar_Project\LigaMX\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72638C44-8595-4505-BEB3-D2CF2ED50218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{872D99E4-723E-44EF-8179-AF39D28DE112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{74EB7EE7-EB5C-4423-87E4-FE46F1C4926A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="899" uniqueCount="95">
   <si>
     <t>Model</t>
   </si>
@@ -307,16 +307,37 @@
   </si>
   <si>
     <t>Final</t>
+  </si>
+  <si>
+    <t>Pumas UNAM Loss</t>
+  </si>
+  <si>
+    <t>Temporada</t>
+  </si>
+  <si>
+    <t>CL26</t>
+  </si>
+  <si>
+    <t>Guadalajara Loss</t>
+  </si>
+  <si>
+    <t>Cruz Azul Loss</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1632,14 +1653,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2AB4D39-76AB-4A8D-8A49-E2E912416120}">
-  <dimension ref="A1:E168"/>
+  <dimension ref="A1:F168"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="2" max="3" width="13.578125" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="17.578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>48</v>
       </c>
@@ -1655,8 +1676,11 @@
       <c r="E1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1672,8 +1696,11 @@
       <c r="E2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1689,8 +1716,11 @@
       <c r="E3" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A4">
         <v>1</v>
       </c>
@@ -1706,8 +1736,11 @@
       <c r="E4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A5">
         <v>1</v>
       </c>
@@ -1723,8 +1756,11 @@
       <c r="E5" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A6">
         <v>1</v>
       </c>
@@ -1740,8 +1776,11 @@
       <c r="E6" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1757,8 +1796,11 @@
       <c r="E7" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A8">
         <v>1</v>
       </c>
@@ -1774,8 +1816,11 @@
       <c r="E8" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A9">
         <v>1</v>
       </c>
@@ -1791,8 +1836,11 @@
       <c r="E9" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A10">
         <v>1</v>
       </c>
@@ -1808,8 +1856,11 @@
       <c r="E10" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A11">
         <v>2</v>
       </c>
@@ -1825,8 +1876,11 @@
       <c r="E11" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F11" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A12">
         <v>2</v>
       </c>
@@ -1842,8 +1896,11 @@
       <c r="E12" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F12" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A13">
         <v>2</v>
       </c>
@@ -1859,8 +1916,11 @@
       <c r="E13" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F13" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A14">
         <v>2</v>
       </c>
@@ -1876,8 +1936,11 @@
       <c r="E14" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F14" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A15">
         <v>2</v>
       </c>
@@ -1893,8 +1956,11 @@
       <c r="E15" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F15" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16">
         <v>2</v>
       </c>
@@ -1910,8 +1976,11 @@
       <c r="E16" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F16" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A17">
         <v>2</v>
       </c>
@@ -1927,8 +1996,11 @@
       <c r="E17" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F17" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A18">
         <v>2</v>
       </c>
@@ -1944,8 +2016,11 @@
       <c r="E18" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F18" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A19">
         <v>2</v>
       </c>
@@ -1961,8 +2036,11 @@
       <c r="E19" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F19" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A20">
         <v>3</v>
       </c>
@@ -1978,8 +2056,11 @@
       <c r="E20" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F20" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A21">
         <v>3</v>
       </c>
@@ -1995,8 +2076,11 @@
       <c r="E21" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F21" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A22">
         <v>3</v>
       </c>
@@ -2012,8 +2096,11 @@
       <c r="E22" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F22" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A23">
         <v>3</v>
       </c>
@@ -2029,8 +2116,11 @@
       <c r="E23" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F23" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A24">
         <v>3</v>
       </c>
@@ -2046,8 +2136,11 @@
       <c r="E24" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F24" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A25">
         <v>3</v>
       </c>
@@ -2063,8 +2156,11 @@
       <c r="E25" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F25" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A26">
         <v>3</v>
       </c>
@@ -2080,8 +2176,11 @@
       <c r="E26" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F26" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A27">
         <v>3</v>
       </c>
@@ -2097,8 +2196,11 @@
       <c r="E27" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F27" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A28">
         <v>3</v>
       </c>
@@ -2114,8 +2216,11 @@
       <c r="E28" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A29">
         <v>4</v>
       </c>
@@ -2131,8 +2236,11 @@
       <c r="E29" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F29" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A30">
         <v>4</v>
       </c>
@@ -2148,8 +2256,11 @@
       <c r="E30" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A31">
         <v>4</v>
       </c>
@@ -2165,8 +2276,11 @@
       <c r="E31" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F31" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A32">
         <v>4</v>
       </c>
@@ -2182,8 +2296,11 @@
       <c r="E32" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F32" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A33">
         <v>4</v>
       </c>
@@ -2199,8 +2316,11 @@
       <c r="E33" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F33" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A34">
         <v>4</v>
       </c>
@@ -2216,8 +2336,11 @@
       <c r="E34" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F34" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A35">
         <v>4</v>
       </c>
@@ -2233,8 +2356,11 @@
       <c r="E35" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F35" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A36">
         <v>4</v>
       </c>
@@ -2250,8 +2376,11 @@
       <c r="E36" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F36" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A37">
         <v>4</v>
       </c>
@@ -2267,8 +2396,11 @@
       <c r="E37" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F37" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A38">
         <v>5</v>
       </c>
@@ -2284,8 +2416,11 @@
       <c r="E38" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F38" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A39">
         <v>5</v>
       </c>
@@ -2301,8 +2436,11 @@
       <c r="E39" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F39" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A40">
         <v>5</v>
       </c>
@@ -2318,8 +2456,11 @@
       <c r="E40" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F40" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A41">
         <v>5</v>
       </c>
@@ -2335,8 +2476,11 @@
       <c r="E41" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A42">
         <v>5</v>
       </c>
@@ -2352,8 +2496,11 @@
       <c r="E42" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F42" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A43">
         <v>5</v>
       </c>
@@ -2369,8 +2516,11 @@
       <c r="E43" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F43" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A44">
         <v>5</v>
       </c>
@@ -2386,8 +2536,11 @@
       <c r="E44" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F44" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A45">
         <v>5</v>
       </c>
@@ -2403,8 +2556,11 @@
       <c r="E45" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F45" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A46">
         <v>5</v>
       </c>
@@ -2420,8 +2576,11 @@
       <c r="E46" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F46" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A47">
         <v>6</v>
       </c>
@@ -2437,8 +2596,11 @@
       <c r="E47" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F47" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A48">
         <v>6</v>
       </c>
@@ -2454,8 +2616,11 @@
       <c r="E48" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F48" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A49">
         <v>6</v>
       </c>
@@ -2471,8 +2636,11 @@
       <c r="E49" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F49" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A50">
         <v>6</v>
       </c>
@@ -2488,8 +2656,11 @@
       <c r="E50" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F50" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A51">
         <v>6</v>
       </c>
@@ -2505,8 +2676,11 @@
       <c r="E51" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F51" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A52">
         <v>6</v>
       </c>
@@ -2522,8 +2696,11 @@
       <c r="E52" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F52" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A53">
         <v>6</v>
       </c>
@@ -2539,8 +2716,11 @@
       <c r="E53" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F53" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A54">
         <v>6</v>
       </c>
@@ -2556,8 +2736,11 @@
       <c r="E54" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F54" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A55">
         <v>6</v>
       </c>
@@ -2573,368 +2756,1451 @@
       <c r="E55" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F55" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A56">
         <v>7</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B56" t="s">
+        <v>53</v>
+      </c>
+      <c r="C56" t="s">
+        <v>24</v>
+      </c>
+      <c r="D56" t="s">
+        <v>71</v>
+      </c>
+      <c r="E56" t="s">
+        <v>71</v>
+      </c>
+      <c r="F56" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A57">
         <v>7</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B57" t="s">
+        <v>30</v>
+      </c>
+      <c r="C57" t="s">
+        <v>36</v>
+      </c>
+      <c r="D57" t="s">
+        <v>47</v>
+      </c>
+      <c r="E57" t="s">
+        <v>77</v>
+      </c>
+      <c r="F57" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A58">
         <v>7</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B58" t="s">
+        <v>27</v>
+      </c>
+      <c r="C58" t="s">
+        <v>49</v>
+      </c>
+      <c r="D58" t="s">
+        <v>69</v>
+      </c>
+      <c r="E58" t="s">
+        <v>69</v>
+      </c>
+      <c r="F58" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A59">
         <v>7</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B59" t="s">
+        <v>25</v>
+      </c>
+      <c r="C59" t="s">
+        <v>35</v>
+      </c>
+      <c r="D59" t="s">
+        <v>90</v>
+      </c>
+      <c r="E59" t="s">
+        <v>58</v>
+      </c>
+      <c r="F59" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A60">
         <v>7</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B60" t="s">
+        <v>43</v>
+      </c>
+      <c r="C60" t="s">
+        <v>52</v>
+      </c>
+      <c r="D60" t="s">
+        <v>45</v>
+      </c>
+      <c r="E60" t="s">
+        <v>45</v>
+      </c>
+      <c r="F60" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A61">
         <v>7</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B61" t="s">
+        <v>29</v>
+      </c>
+      <c r="C61" t="s">
+        <v>50</v>
+      </c>
+      <c r="D61" t="s">
+        <v>31</v>
+      </c>
+      <c r="E61" t="s">
+        <v>31</v>
+      </c>
+      <c r="F61" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A62">
         <v>7</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B62" t="s">
+        <v>32</v>
+      </c>
+      <c r="C62" t="s">
+        <v>39</v>
+      </c>
+      <c r="D62" t="s">
+        <v>34</v>
+      </c>
+      <c r="E62" t="s">
+        <v>34</v>
+      </c>
+      <c r="F62" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A63">
         <v>7</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B63" t="s">
+        <v>33</v>
+      </c>
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63" t="s">
+        <v>66</v>
+      </c>
+      <c r="E63" t="s">
+        <v>47</v>
+      </c>
+      <c r="F63" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A64">
         <v>7</v>
       </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B64" t="s">
+        <v>38</v>
+      </c>
+      <c r="C64" t="s">
+        <v>44</v>
+      </c>
+      <c r="D64" t="s">
+        <v>81</v>
+      </c>
+      <c r="E64" t="s">
+        <v>47</v>
+      </c>
+      <c r="F64" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A65">
         <v>8</v>
       </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B65" t="s">
+        <v>24</v>
+      </c>
+      <c r="C65" t="s">
+        <v>27</v>
+      </c>
+      <c r="D65" t="s">
+        <v>63</v>
+      </c>
+      <c r="E65" t="s">
+        <v>64</v>
+      </c>
+      <c r="F65" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A66">
         <v>8</v>
       </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B66" t="s">
+        <v>50</v>
+      </c>
+      <c r="C66" t="s">
+        <v>39</v>
+      </c>
+      <c r="D66" t="s">
+        <v>78</v>
+      </c>
+      <c r="E66" t="s">
+        <v>78</v>
+      </c>
+      <c r="F66" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A67">
         <v>8</v>
       </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B67" t="s">
+        <v>26</v>
+      </c>
+      <c r="C67" t="s">
+        <v>36</v>
+      </c>
+      <c r="D67" t="s">
+        <v>65</v>
+      </c>
+      <c r="E67" t="s">
+        <v>28</v>
+      </c>
+      <c r="F67" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A68">
         <v>8</v>
       </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B68" t="s">
+        <v>38</v>
+      </c>
+      <c r="C68" t="s">
+        <v>52</v>
+      </c>
+      <c r="D68" t="s">
+        <v>81</v>
+      </c>
+      <c r="E68" t="s">
+        <v>47</v>
+      </c>
+      <c r="F68" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A69">
         <v>8</v>
       </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B69" t="s">
+        <v>33</v>
+      </c>
+      <c r="C69" t="s">
+        <v>25</v>
+      </c>
+      <c r="D69" t="s">
+        <v>66</v>
+      </c>
+      <c r="E69" t="s">
+        <v>47</v>
+      </c>
+      <c r="F69" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A70">
         <v>8</v>
       </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B70" t="s">
+        <v>44</v>
+      </c>
+      <c r="C70" t="s">
+        <v>53</v>
+      </c>
+      <c r="D70" t="s">
+        <v>47</v>
+      </c>
+      <c r="E70" t="s">
+        <v>83</v>
+      </c>
+      <c r="F70" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A71">
         <v>8</v>
       </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B71" t="s">
+        <v>35</v>
+      </c>
+      <c r="C71" t="s">
+        <v>32</v>
+      </c>
+      <c r="D71" t="s">
+        <v>46</v>
+      </c>
+      <c r="E71" t="s">
+        <v>46</v>
+      </c>
+      <c r="F71" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A72">
         <v>8</v>
       </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B72" t="s">
+        <v>43</v>
+      </c>
+      <c r="C72" t="s">
+        <v>29</v>
+      </c>
+      <c r="D72" t="s">
+        <v>45</v>
+      </c>
+      <c r="E72" t="s">
+        <v>45</v>
+      </c>
+      <c r="F72" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A73">
         <v>8</v>
       </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B73" t="s">
+        <v>49</v>
+      </c>
+      <c r="C73" t="s">
+        <v>30</v>
+      </c>
+      <c r="D73" t="s">
+        <v>75</v>
+      </c>
+      <c r="E73" t="s">
+        <v>75</v>
+      </c>
+      <c r="F73" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A74">
         <v>9</v>
       </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B74" t="s">
+        <v>36</v>
+      </c>
+      <c r="C74" t="s">
+        <v>29</v>
+      </c>
+      <c r="D74" t="s">
+        <v>73</v>
+      </c>
+      <c r="E74" t="s">
+        <v>73</v>
+      </c>
+      <c r="F74" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A75">
         <v>9</v>
       </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B75" t="s">
+        <v>52</v>
+      </c>
+      <c r="C75" t="s">
+        <v>32</v>
+      </c>
+      <c r="D75" t="s">
+        <v>54</v>
+      </c>
+      <c r="E75" t="s">
+        <v>54</v>
+      </c>
+      <c r="F75" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A76">
         <v>9</v>
       </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B76" t="s">
+        <v>24</v>
+      </c>
+      <c r="C76" t="s">
+        <v>26</v>
+      </c>
+      <c r="D76" t="s">
+        <v>63</v>
+      </c>
+      <c r="E76" t="s">
+        <v>63</v>
+      </c>
+      <c r="F76" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A77">
         <v>9</v>
       </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B77" t="s">
+        <v>25</v>
+      </c>
+      <c r="C77" t="s">
+        <v>50</v>
+      </c>
+      <c r="D77" t="s">
+        <v>47</v>
+      </c>
+      <c r="E77" t="s">
+        <v>90</v>
+      </c>
+      <c r="F77" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A78">
         <v>9</v>
       </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B78" t="s">
+        <v>27</v>
+      </c>
+      <c r="C78" t="s">
+        <v>30</v>
+      </c>
+      <c r="D78" t="s">
+        <v>69</v>
+      </c>
+      <c r="E78" t="s">
+        <v>72</v>
+      </c>
+      <c r="F78" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A79">
         <v>9</v>
       </c>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B79" t="s">
+        <v>35</v>
+      </c>
+      <c r="C79" t="s">
+        <v>38</v>
+      </c>
+      <c r="D79" t="s">
+        <v>37</v>
+      </c>
+      <c r="E79" t="s">
+        <v>37</v>
+      </c>
+      <c r="F79" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A80">
         <v>9</v>
       </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B80" t="s">
+        <v>53</v>
+      </c>
+      <c r="C80" t="s">
+        <v>33</v>
+      </c>
+      <c r="D80" t="s">
+        <v>62</v>
+      </c>
+      <c r="E80" t="s">
+        <v>71</v>
+      </c>
+      <c r="F80" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A81">
         <v>9</v>
       </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B81" t="s">
+        <v>49</v>
+      </c>
+      <c r="C81" t="s">
+        <v>44</v>
+      </c>
+      <c r="D81" t="s">
+        <v>51</v>
+      </c>
+      <c r="E81" t="s">
+        <v>75</v>
+      </c>
+      <c r="F81" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A82">
         <v>9</v>
       </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B82" t="s">
+        <v>39</v>
+      </c>
+      <c r="C82" t="s">
+        <v>43</v>
+      </c>
+      <c r="D82" t="s">
+        <v>40</v>
+      </c>
+      <c r="E82" t="s">
+        <v>40</v>
+      </c>
+      <c r="F82" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A83">
         <v>10</v>
       </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B83" t="s">
+        <v>32</v>
+      </c>
+      <c r="C83" t="s">
+        <v>24</v>
+      </c>
+      <c r="D83" t="s">
+        <v>34</v>
+      </c>
+      <c r="E83" t="s">
+        <v>34</v>
+      </c>
+      <c r="F83" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A84">
         <v>10</v>
       </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B84" t="s">
+        <v>38</v>
+      </c>
+      <c r="C84" t="s">
+        <v>49</v>
+      </c>
+      <c r="D84" t="s">
+        <v>59</v>
+      </c>
+      <c r="E84" t="s">
+        <v>59</v>
+      </c>
+      <c r="F84" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A85">
         <v>10</v>
       </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B85" t="s">
+        <v>26</v>
+      </c>
+      <c r="C85" t="s">
+        <v>43</v>
+      </c>
+      <c r="D85" t="s">
+        <v>65</v>
+      </c>
+      <c r="E85" t="s">
+        <v>28</v>
+      </c>
+      <c r="F85" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A86">
         <v>10</v>
       </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B86" t="s">
+        <v>29</v>
+      </c>
+      <c r="C86" t="s">
+        <v>25</v>
+      </c>
+      <c r="D86" t="s">
+        <v>79</v>
+      </c>
+      <c r="E86" t="s">
+        <v>31</v>
+      </c>
+      <c r="F86" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A87">
         <v>10</v>
       </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B87" t="s">
+        <v>50</v>
+      </c>
+      <c r="C87" t="s">
+        <v>44</v>
+      </c>
+      <c r="D87" t="s">
+        <v>78</v>
+      </c>
+      <c r="E87" t="s">
+        <v>78</v>
+      </c>
+      <c r="F87" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A88">
         <v>10</v>
       </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B88" t="s">
+        <v>53</v>
+      </c>
+      <c r="C88" t="s">
+        <v>39</v>
+      </c>
+      <c r="D88" t="s">
+        <v>62</v>
+      </c>
+      <c r="E88" t="s">
+        <v>62</v>
+      </c>
+      <c r="F88" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A89">
         <v>10</v>
       </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B89" t="s">
+        <v>36</v>
+      </c>
+      <c r="C89" t="s">
+        <v>27</v>
+      </c>
+      <c r="D89" t="s">
+        <v>73</v>
+      </c>
+      <c r="E89" t="s">
+        <v>73</v>
+      </c>
+      <c r="F89" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A90">
         <v>10</v>
       </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B90" t="s">
+        <v>30</v>
+      </c>
+      <c r="C90" t="s">
+        <v>35</v>
+      </c>
+      <c r="D90" t="s">
+        <v>76</v>
+      </c>
+      <c r="E90" t="s">
+        <v>76</v>
+      </c>
+      <c r="F90" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A91">
         <v>10</v>
       </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B91" t="s">
+        <v>33</v>
+      </c>
+      <c r="C91" t="s">
+        <v>52</v>
+      </c>
+      <c r="D91" t="s">
+        <v>66</v>
+      </c>
+      <c r="E91" t="s">
+        <v>70</v>
+      </c>
+      <c r="F91" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A92">
         <v>11</v>
       </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B92" t="s">
+        <v>24</v>
+      </c>
+      <c r="C92" t="s">
+        <v>36</v>
+      </c>
+      <c r="D92" t="s">
+        <v>64</v>
+      </c>
+      <c r="E92" t="s">
+        <v>47</v>
+      </c>
+      <c r="F92" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A93">
         <v>11</v>
       </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B93" t="s">
+        <v>39</v>
+      </c>
+      <c r="C93" t="s">
+        <v>52</v>
+      </c>
+      <c r="D93" t="s">
+        <v>40</v>
+      </c>
+      <c r="E93" t="s">
+        <v>40</v>
+      </c>
+      <c r="F93" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A94">
         <v>11</v>
       </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B94" t="s">
+        <v>27</v>
+      </c>
+      <c r="C94" t="s">
+        <v>29</v>
+      </c>
+      <c r="D94" t="s">
+        <v>69</v>
+      </c>
+      <c r="E94" t="s">
+        <v>47</v>
+      </c>
+      <c r="F94" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A95">
         <v>11</v>
       </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B95" t="s">
+        <v>44</v>
+      </c>
+      <c r="C95" t="s">
+        <v>35</v>
+      </c>
+      <c r="D95" t="s">
+        <v>74</v>
+      </c>
+      <c r="E95" t="s">
+        <v>47</v>
+      </c>
+      <c r="F95" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A96">
         <v>11</v>
       </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B96" t="s">
+        <v>30</v>
+      </c>
+      <c r="C96" t="s">
+        <v>38</v>
+      </c>
+      <c r="D96" t="s">
+        <v>76</v>
+      </c>
+      <c r="E96" t="s">
+        <v>47</v>
+      </c>
+      <c r="F96" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A97">
         <v>11</v>
       </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B97" t="s">
+        <v>43</v>
+      </c>
+      <c r="C97" t="s">
+        <v>33</v>
+      </c>
+      <c r="D97" t="s">
+        <v>45</v>
+      </c>
+      <c r="E97" t="s">
+        <v>61</v>
+      </c>
+      <c r="F97" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A98">
         <v>11</v>
       </c>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B98" t="s">
+        <v>50</v>
+      </c>
+      <c r="C98" t="s">
+        <v>53</v>
+      </c>
+      <c r="D98" t="s">
+        <v>78</v>
+      </c>
+      <c r="E98" t="s">
+        <v>47</v>
+      </c>
+      <c r="F98" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A99">
         <v>11</v>
       </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B99" t="s">
+        <v>25</v>
+      </c>
+      <c r="C99" t="s">
+        <v>32</v>
+      </c>
+      <c r="D99" t="s">
+        <v>90</v>
+      </c>
+      <c r="E99" t="s">
+        <v>47</v>
+      </c>
+      <c r="F99" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A100">
         <v>11</v>
       </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B100" t="s">
+        <v>49</v>
+      </c>
+      <c r="C100" t="s">
+        <v>26</v>
+      </c>
+      <c r="D100" t="s">
+        <v>51</v>
+      </c>
+      <c r="E100" t="s">
+        <v>51</v>
+      </c>
+      <c r="F100" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A101">
         <v>12</v>
       </c>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B101" t="s">
+        <v>53</v>
+      </c>
+      <c r="C101" t="s">
+        <v>38</v>
+      </c>
+      <c r="D101" t="s">
+        <v>71</v>
+      </c>
+      <c r="E101" t="s">
+        <v>47</v>
+      </c>
+      <c r="F101" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A102">
         <v>12</v>
       </c>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B102" t="s">
+        <v>29</v>
+      </c>
+      <c r="C102" t="s">
+        <v>33</v>
+      </c>
+      <c r="D102" t="s">
+        <v>79</v>
+      </c>
+      <c r="E102" t="s">
+        <v>79</v>
+      </c>
+      <c r="F102" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A103">
         <v>12</v>
       </c>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B103" t="s">
+        <v>26</v>
+      </c>
+      <c r="C103" t="s">
+        <v>32</v>
+      </c>
+      <c r="D103" t="s">
+        <v>65</v>
+      </c>
+      <c r="E103" t="s">
+        <v>47</v>
+      </c>
+      <c r="F103" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A104">
         <v>12</v>
       </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B104" t="s">
+        <v>52</v>
+      </c>
+      <c r="C104" t="s">
+        <v>27</v>
+      </c>
+      <c r="D104" t="s">
+        <v>85</v>
+      </c>
+      <c r="E104" t="s">
+        <v>85</v>
+      </c>
+      <c r="F104" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A105">
         <v>12</v>
       </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B105" t="s">
+        <v>36</v>
+      </c>
+      <c r="C105" t="s">
+        <v>50</v>
+      </c>
+      <c r="D105" t="s">
+        <v>73</v>
+      </c>
+      <c r="E105" t="s">
+        <v>47</v>
+      </c>
+      <c r="F105" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A106">
         <v>12</v>
       </c>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B106" t="s">
+        <v>24</v>
+      </c>
+      <c r="C106" t="s">
+        <v>43</v>
+      </c>
+      <c r="D106" t="s">
+        <v>63</v>
+      </c>
+      <c r="E106" t="s">
+        <v>64</v>
+      </c>
+      <c r="F106" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A107">
         <v>12</v>
       </c>
-    </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B107" t="s">
+        <v>35</v>
+      </c>
+      <c r="C107" t="s">
+        <v>39</v>
+      </c>
+      <c r="D107" t="s">
+        <v>46</v>
+      </c>
+      <c r="E107" t="s">
+        <v>46</v>
+      </c>
+      <c r="F107" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A108">
         <v>12</v>
       </c>
-    </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B108" t="s">
+        <v>25</v>
+      </c>
+      <c r="C108" t="s">
+        <v>49</v>
+      </c>
+      <c r="D108" t="s">
+        <v>58</v>
+      </c>
+      <c r="E108" t="s">
+        <v>58</v>
+      </c>
+      <c r="F108" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A109">
         <v>12</v>
       </c>
-    </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B109" t="s">
+        <v>44</v>
+      </c>
+      <c r="C109" t="s">
+        <v>30</v>
+      </c>
+      <c r="D109" t="s">
+        <v>74</v>
+      </c>
+      <c r="E109" t="s">
+        <v>83</v>
+      </c>
+      <c r="F109" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A110">
         <v>13</v>
       </c>
-    </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B110" t="s">
+        <v>38</v>
+      </c>
+      <c r="C110" t="s">
+        <v>50</v>
+      </c>
+      <c r="D110" t="s">
+        <v>59</v>
+      </c>
+      <c r="E110" t="s">
+        <v>81</v>
+      </c>
+      <c r="F110" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A111">
         <v>13</v>
       </c>
-    </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B111" t="s">
+        <v>35</v>
+      </c>
+      <c r="C111" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111" t="s">
+        <v>37</v>
+      </c>
+      <c r="E111" t="s">
+        <v>46</v>
+      </c>
+      <c r="F111" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A112">
         <v>13</v>
       </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B112" t="s">
+        <v>27</v>
+      </c>
+      <c r="C112" t="s">
+        <v>44</v>
+      </c>
+      <c r="D112" t="s">
+        <v>69</v>
+      </c>
+      <c r="E112" t="s">
+        <v>47</v>
+      </c>
+      <c r="F112" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A113">
         <v>13</v>
       </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B113" t="s">
+        <v>33</v>
+      </c>
+      <c r="C113" t="s">
+        <v>30</v>
+      </c>
+      <c r="D113" t="s">
+        <v>47</v>
+      </c>
+      <c r="E113" t="s">
+        <v>66</v>
+      </c>
+      <c r="F113" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A114">
         <v>13</v>
       </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B114" t="s">
+        <v>29</v>
+      </c>
+      <c r="C114" t="s">
+        <v>26</v>
+      </c>
+      <c r="D114" t="s">
+        <v>79</v>
+      </c>
+      <c r="E114" t="s">
+        <v>79</v>
+      </c>
+      <c r="F114" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A115">
         <v>13</v>
       </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B115" t="s">
+        <v>43</v>
+      </c>
+      <c r="C115" t="s">
+        <v>53</v>
+      </c>
+      <c r="D115" t="s">
+        <v>45</v>
+      </c>
+      <c r="E115" t="s">
+        <v>45</v>
+      </c>
+      <c r="F115" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A116">
         <v>13</v>
       </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B116" t="s">
+        <v>32</v>
+      </c>
+      <c r="C116" t="s">
+        <v>36</v>
+      </c>
+      <c r="D116" t="s">
+        <v>34</v>
+      </c>
+      <c r="E116" t="s">
+        <v>94</v>
+      </c>
+      <c r="F116" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A117">
         <v>13</v>
       </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B117" t="s">
+        <v>52</v>
+      </c>
+      <c r="C117" t="s">
+        <v>49</v>
+      </c>
+      <c r="D117" t="s">
+        <v>54</v>
+      </c>
+      <c r="E117" t="s">
+        <v>47</v>
+      </c>
+      <c r="F117" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A118">
         <v>13</v>
       </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B118" t="s">
+        <v>39</v>
+      </c>
+      <c r="C118" t="s">
+        <v>25</v>
+      </c>
+      <c r="D118" t="s">
+        <v>93</v>
+      </c>
+      <c r="E118" t="s">
+        <v>47</v>
+      </c>
+      <c r="F118" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A119">
         <v>14</v>
       </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B119" t="s">
+        <v>38</v>
+      </c>
+      <c r="C119" t="s">
+        <v>29</v>
+      </c>
+      <c r="D119" t="s">
+        <v>81</v>
+      </c>
+      <c r="E119" t="s">
+        <v>81</v>
+      </c>
+      <c r="F119" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A120">
         <v>14</v>
       </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B120" t="s">
+        <v>30</v>
+      </c>
+      <c r="C120" t="s">
+        <v>39</v>
+      </c>
+      <c r="D120" t="s">
+        <v>76</v>
+      </c>
+      <c r="E120" t="s">
+        <v>76</v>
+      </c>
+      <c r="F120" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A121">
         <v>14</v>
       </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B121" t="s">
+        <v>27</v>
+      </c>
+      <c r="C121" t="s">
+        <v>43</v>
+      </c>
+      <c r="D121" t="s">
+        <v>69</v>
+      </c>
+      <c r="E121" t="s">
+        <v>69</v>
+      </c>
+      <c r="F121" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A122">
         <v>14</v>
       </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B122" t="s">
+        <v>44</v>
+      </c>
+      <c r="C122" t="s">
+        <v>33</v>
+      </c>
+      <c r="D122" t="s">
+        <v>74</v>
+      </c>
+      <c r="E122" t="s">
+        <v>74</v>
+      </c>
+      <c r="F122" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A123">
         <v>14</v>
       </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B123" t="s">
+        <v>25</v>
+      </c>
+      <c r="C123" t="s">
+        <v>26</v>
+      </c>
+      <c r="D123" t="s">
+        <v>58</v>
+      </c>
+      <c r="E123" t="s">
+        <v>58</v>
+      </c>
+      <c r="F123" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A124">
         <v>14</v>
       </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B124" t="s">
+        <v>36</v>
+      </c>
+      <c r="C124" t="s">
+        <v>52</v>
+      </c>
+      <c r="D124" t="s">
+        <v>73</v>
+      </c>
+      <c r="E124" t="s">
+        <v>73</v>
+      </c>
+      <c r="F124" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A125">
         <v>14</v>
       </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B125" t="s">
+        <v>53</v>
+      </c>
+      <c r="C125" t="s">
+        <v>35</v>
+      </c>
+      <c r="D125" t="s">
+        <v>62</v>
+      </c>
+      <c r="E125" t="s">
+        <v>47</v>
+      </c>
+      <c r="F125" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A126">
         <v>14</v>
       </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B126" t="s">
+        <v>49</v>
+      </c>
+      <c r="C126" t="s">
+        <v>32</v>
+      </c>
+      <c r="D126" t="s">
+        <v>51</v>
+      </c>
+      <c r="E126" t="s">
+        <v>47</v>
+      </c>
+      <c r="F126" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A127">
         <v>14</v>
       </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B127" t="s">
+        <v>50</v>
+      </c>
+      <c r="C127" t="s">
+        <v>24</v>
+      </c>
+      <c r="D127" t="s">
+        <v>78</v>
+      </c>
+      <c r="E127" t="s">
+        <v>47</v>
+      </c>
+      <c r="F127" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A128">
         <v>15</v>
       </c>
@@ -2950,8 +4216,11 @@
       <c r="E128" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F128" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A129">
         <v>15</v>
       </c>
@@ -2967,8 +4236,11 @@
       <c r="E129" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F129" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A130">
         <v>15</v>
       </c>
@@ -2984,8 +4256,11 @@
       <c r="E130" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F130" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A131">
         <v>15</v>
       </c>
@@ -3001,8 +4276,11 @@
       <c r="E131" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F131" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A132">
         <v>15</v>
       </c>
@@ -3018,8 +4296,11 @@
       <c r="E132" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F132" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A133">
         <v>15</v>
       </c>
@@ -3035,8 +4316,11 @@
       <c r="E133" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F133" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A134">
         <v>15</v>
       </c>
@@ -3052,8 +4336,11 @@
       <c r="E134" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F134" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A135">
         <v>15</v>
       </c>
@@ -3069,8 +4356,11 @@
       <c r="E135" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F135" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A136">
         <v>15</v>
       </c>
@@ -3086,8 +4376,11 @@
       <c r="E136" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F136" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A137">
         <v>16</v>
       </c>
@@ -3103,8 +4396,11 @@
       <c r="E137" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F137" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A138">
         <v>16</v>
       </c>
@@ -3120,8 +4416,11 @@
       <c r="E138" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F138" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A139">
         <v>16</v>
       </c>
@@ -3137,8 +4436,11 @@
       <c r="E139" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F139" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A140">
         <v>16</v>
       </c>
@@ -3154,8 +4456,11 @@
       <c r="E140" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F140" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A141">
         <v>16</v>
       </c>
@@ -3171,8 +4476,11 @@
       <c r="E141" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F141" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A142">
         <v>16</v>
       </c>
@@ -3188,8 +4496,11 @@
       <c r="E142" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F142" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A143">
         <v>16</v>
       </c>
@@ -3205,8 +4516,11 @@
       <c r="E143" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F143" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A144">
         <v>16</v>
       </c>
@@ -3222,8 +4536,11 @@
       <c r="E144" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F144" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A145">
         <v>16</v>
       </c>
@@ -3239,8 +4556,11 @@
       <c r="E145" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F145" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A146">
         <v>17</v>
       </c>
@@ -3256,8 +4576,11 @@
       <c r="E146" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F146" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A147">
         <v>17</v>
       </c>
@@ -3273,8 +4596,11 @@
       <c r="E147" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F147" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A148">
         <v>17</v>
       </c>
@@ -3290,8 +4616,11 @@
       <c r="E148" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F148" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A149">
         <v>17</v>
       </c>
@@ -3307,8 +4636,11 @@
       <c r="E149" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F149" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A150">
         <v>17</v>
       </c>
@@ -3324,8 +4656,11 @@
       <c r="E150" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F150" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A151">
         <v>17</v>
       </c>
@@ -3341,8 +4676,11 @@
       <c r="E151" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F151" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A152">
         <v>17</v>
       </c>
@@ -3358,8 +4696,11 @@
       <c r="E152" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F152" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A153">
         <v>17</v>
       </c>
@@ -3375,8 +4716,11 @@
       <c r="E153" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F153" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A154">
         <v>17</v>
       </c>
@@ -3392,8 +4736,11 @@
       <c r="E154" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F154" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A155" t="s">
         <v>86</v>
       </c>
@@ -3409,8 +4756,11 @@
       <c r="E155" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F155" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A156" t="s">
         <v>86</v>
       </c>
@@ -3426,8 +4776,11 @@
       <c r="E156" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F156" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A157" t="s">
         <v>86</v>
       </c>
@@ -3443,8 +4796,11 @@
       <c r="E157" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F157" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A158" t="s">
         <v>86</v>
       </c>
@@ -3460,8 +4816,11 @@
       <c r="E158" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F158" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A159" t="s">
         <v>86</v>
       </c>
@@ -3477,8 +4836,11 @@
       <c r="E159" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F159" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A160" t="s">
         <v>86</v>
       </c>
@@ -3494,8 +4856,11 @@
       <c r="E160" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F160" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A161" t="s">
         <v>86</v>
       </c>
@@ -3511,8 +4876,11 @@
       <c r="E161" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F161" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A162" t="s">
         <v>86</v>
       </c>
@@ -3528,8 +4896,11 @@
       <c r="E162" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F162" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A163" t="s">
         <v>88</v>
       </c>
@@ -3545,8 +4916,11 @@
       <c r="E163" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F163" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A164" t="s">
         <v>88</v>
       </c>
@@ -3562,8 +4936,11 @@
       <c r="E164" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F164" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A165" t="s">
         <v>88</v>
       </c>
@@ -3579,8 +4956,11 @@
       <c r="E165" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F165" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A166" t="s">
         <v>88</v>
       </c>
@@ -3596,18 +4976,52 @@
       <c r="E166" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="F166" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A167" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B167" t="s">
+        <v>32</v>
+      </c>
+      <c r="C167" t="s">
+        <v>25</v>
+      </c>
+      <c r="D167" t="s">
+        <v>34</v>
+      </c>
+      <c r="E167" t="s">
+        <v>47</v>
+      </c>
+      <c r="F167" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A168" t="s">
         <v>89</v>
       </c>
+      <c r="B168" t="s">
+        <v>25</v>
+      </c>
+      <c r="C168" t="s">
+        <v>32</v>
+      </c>
+      <c r="D168" t="s">
+        <v>90</v>
+      </c>
+      <c r="E168" t="s">
+        <v>90</v>
+      </c>
+      <c r="F168" t="s">
+        <v>92</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>